<commit_message>
Pre-fill забор/распродажа registry with 66 SKU from plan (Ozon pull, WB liquidate, WB targeted pull)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RB3ZzCvNjh49PbwKyrmhRr
</commit_message>
<xml_diff>
--- a/Таблицы/Шаблон_замера_локализации.xlsx
+++ b/Таблицы/Шаблон_замера_локализации.xlsx
@@ -18,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0 ₽"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +43,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +62,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,6 +123,42 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1162,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1225,409 +1281,2280 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>D212</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Клевер»</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>D274</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Листики»</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>420</v>
+      </c>
+      <c r="G5" s="8" t="inlineStr"/>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>D249</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Капли»</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>330</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>D354</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Ракушки»</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-039</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Найтли»</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>300</v>
+      </c>
+      <c r="G8" s="8" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>MSH-074</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Эстелла»</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>270</v>
+      </c>
+      <c r="G9" s="8" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>D159</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Скарабеи»</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="G10" s="8" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-037</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Габриэль»</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>D531</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Доминика»</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="G12" s="8" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-028</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Колье «Алма»</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G13" s="8" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>D388</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Листва»</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G14" s="8" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>D542</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо «Анемон»</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G15" s="8" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>D355</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Рыбки»</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G16" s="8" t="inlineStr"/>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>MSH-082</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Сабрина»</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G17" s="8" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>D512</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Афина»</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-045</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Зои»</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G19" s="8" t="inlineStr"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>D535</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Камилла»</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>MSH-073</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Матильда»</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>MSH-083</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Сабрина»</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>D529</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо «Ирис»</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G23" s="8" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>D519</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Весенние тюльпаны»</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G24" s="8" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>D236</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Цикада»</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>210</v>
+      </c>
+      <c r="G25" s="8" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>MSH-007</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Исидора»</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>D364</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Кэрри»</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G27" s="8" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>D528</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо «Ирис»</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>D495</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо «Роза»</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G29" s="8" t="inlineStr"/>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="n"/>
-      <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>D513</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Афина»</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G30" s="8" t="inlineStr"/>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-055</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Эмма»</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G31" s="8" t="inlineStr"/>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="n"/>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>D216</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Колибри»</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G32" s="8" t="inlineStr"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n"/>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>MSH-002</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Египетские скарабеи»</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G33" s="8" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n"/>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>D527</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Кольцо «Ирис»</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G34" s="8" t="inlineStr"/>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n"/>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>MSH-096</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Валерия»</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G35" s="8" t="inlineStr"/>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n"/>
-      <c r="B36" s="5" t="n"/>
-      <c r="C36" s="5" t="n"/>
-      <c r="D36" s="5" t="n"/>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>MSH-078</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Жанин»</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G36" s="8" t="inlineStr"/>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>MSH-013</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Лучиана»</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G37" s="8" t="inlineStr"/>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n"/>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>MSH-026</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Алисия»</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n"/>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>D518</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Тропики»</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="G39" s="8" t="inlineStr"/>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n"/>
-      <c r="B40" s="5" t="n"/>
-      <c r="C40" s="5" t="n"/>
-      <c r="D40" s="5" t="n"/>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>D292</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Винтаж»</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="G40" s="8" t="inlineStr"/>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n"/>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>D117</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Сережки ассиметричные «Змеи»</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="G41" s="8" t="inlineStr"/>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n"/>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>MSH-065</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Агнес»</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="G42" s="8" t="inlineStr"/>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n"/>
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="5" t="n"/>
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>MSHK-029</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Колье «Счастливое число 7»</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G43" s="8" t="inlineStr"/>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>D360</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Звездочки»</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Ставки забора: WB 230 ₽/шт, Ozon 30 ₽/шт (товар возвращается для перепродажи)</t>
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>D507-S</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Сережки ассиметричные «Змеи»</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G45" s="8" t="inlineStr"/>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>D523</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «День и ночь»</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G46" s="8" t="inlineStr"/>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>D491</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Катарина»</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G47" s="8" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>MSH-094</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Лора»</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>MSH-097</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Сережки «Тайна сердца»</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Ozon</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="G49" s="8" t="inlineStr"/>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>MSHK-039</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Найтли»</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="F50" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="12" t="inlineStr"/>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>MSH-072</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Барбара»</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F51" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="12" t="inlineStr"/>
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>MSH-013</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Лучиана»</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="F52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="12" t="inlineStr"/>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>MSH-073</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Матильда»</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F53" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="12" t="inlineStr"/>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>MSH-065</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Агнес»</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="12" t="inlineStr"/>
+      <c r="H54" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>MSH-025</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Лаура»</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E55" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="F55" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="12" t="inlineStr"/>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>D175DSR035</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Клевер»</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="12" t="inlineStr"/>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>MSH-012</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Лучиана»</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="12" t="inlineStr"/>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>D513</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Афина»</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F58" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="12" t="inlineStr"/>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>D175DSR098</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Нежный клевер»</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E59" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F59" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="12" t="inlineStr"/>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>MSHK-037</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Габриэль»</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F60" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="12" t="inlineStr"/>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>MSHK-036</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Сильвия»</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F61" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="12" t="inlineStr"/>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>MSH-074</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Эстелла»</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F62" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="12" t="inlineStr"/>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>MSH-070</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Марго»</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E63" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F63" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="12" t="inlineStr"/>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>D175DSR034</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Клевер»</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F64" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="12" t="inlineStr"/>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>MSH-014</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Азалия»</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="12" t="inlineStr"/>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>D193DSR047</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Сережки «Ника»</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>Распродать</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F66" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="12" t="inlineStr"/>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>D114DSMR034</t>
+        </is>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>Моносережка «Перо»</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F67" s="17" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G67" s="15" t="inlineStr"/>
+      <c r="H67" s="15" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>D493</t>
+        </is>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>Сережки «Глаза»</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F68" s="17" t="n">
+        <v>920</v>
+      </c>
+      <c r="G68" s="15" t="inlineStr"/>
+      <c r="H68" s="15" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>D202DSR069-S</t>
+        </is>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>Сережки «Змеи»</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Забрать</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" s="17" t="n">
+        <v>920</v>
+      </c>
+      <c r="G69" s="15" t="inlineStr"/>
+      <c r="H69" s="15" t="inlineStr">
+        <is>
+          <t>Запланировано</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n"/>
+      <c r="C71" s="5" t="n"/>
+      <c r="D71" s="5" t="n"/>
+      <c r="E71" s="18">
+        <f>SUM(E4:E69)</f>
+        <v/>
+      </c>
+      <c r="F71" s="19">
+        <f>SUM(F4:F69)</f>
+        <v/>
+      </c>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Ставки: WB 230 ₽/шт, Ozon 30 ₽/шт (товар возвращается для перепродажи). Распродажа/списание — забор 0 ₽.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Оранжевый — Ozon забрать (мёртвый неликвид) · Зелёный — WB распродать · Жёлтый — WB забрать (дорогой L1).</t>
         </is>
       </c>
     </row>

</xml_diff>